<commit_message>
feat: address reverse causality feedback — early-game controls, skill proxy, extended models
Implements Philippe's feedback on endogeneity / reverse causality:

- build_variables.py: extract early-game fields (CS@10, gold advantage,
  early takedowns) and mechanical skill proxy (solo kills, skillshots)
  from the challenges object in raw match JSONs
- analysis.py: run baseline vs extended logistic regression, add
  close-games robustness check (gold diff < 5k), model comparison
  table and D6 forest plot, updated diagnostics with new variables
- generate_codebook.py: add entries for 4 new variables
- generate_summary.py: new script producing Summary_for_Coworker.docx
  with full methodology, results, embedded figures, and remaining-work
  notes for the paper writer
- .gitignore: exclude zip archives

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Analysis/tables/B1_descriptive_by_region.xlsx
+++ b/Analysis/tables/B1_descriptive_by_region.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EW7"/>
+  <dimension ref="A1:GC7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,6 +510,26 @@
       </c>
       <c r="EP1" t="inlineStr">
         <is>
+          <t>team_early_cs_10</t>
+        </is>
+      </c>
+      <c r="EX1" t="inlineStr">
+        <is>
+          <t>team_early_gold_adv</t>
+        </is>
+      </c>
+      <c r="FF1" t="inlineStr">
+        <is>
+          <t>team_early_takedowns</t>
+        </is>
+      </c>
+      <c r="FN1" t="inlineStr">
+        <is>
+          <t>avg_skill_index</t>
+        </is>
+      </c>
+      <c r="FV1" t="inlineStr">
+        <is>
           <t>win</t>
         </is>
       </c>
@@ -1276,6 +1296,166 @@
           <t>max</t>
         </is>
       </c>
+      <c r="EX2" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="EY2" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="EZ2" t="inlineStr">
+        <is>
+          <t>std</t>
+        </is>
+      </c>
+      <c r="FA2" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="FB2" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="FC2" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="FD2" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="FE2" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="FF2" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="FG2" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="FH2" t="inlineStr">
+        <is>
+          <t>std</t>
+        </is>
+      </c>
+      <c r="FI2" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="FJ2" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="FK2" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="FL2" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="FM2" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="FN2" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="FO2" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="FP2" t="inlineStr">
+        <is>
+          <t>std</t>
+        </is>
+      </c>
+      <c r="FQ2" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="FR2" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="FS2" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="FT2" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="FU2" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="FV2" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="FW2" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="FX2" t="inlineStr">
+        <is>
+          <t>std</t>
+        </is>
+      </c>
+      <c r="FY2" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="FZ2" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="GA2" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="GB2" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="GC2" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1726,24 +1906,120 @@
         <v>4870</v>
       </c>
       <c r="EQ4" t="n">
+        <v>273.5746818016748</v>
+      </c>
+      <c r="ER4" t="n">
+        <v>25.80219457688779</v>
+      </c>
+      <c r="ES4" t="n">
+        <v>182.5000000596046</v>
+      </c>
+      <c r="ET4" t="n">
+        <v>256.000000089407</v>
+      </c>
+      <c r="EU4" t="n">
+        <v>273.2000000923872</v>
+      </c>
+      <c r="EV4" t="n">
+        <v>291.000000089407</v>
+      </c>
+      <c r="EW4" t="n">
+        <v>379.000000089407</v>
+      </c>
+      <c r="EX4" t="n">
+        <v>4870</v>
+      </c>
+      <c r="EY4" t="n">
+        <v>0.07872689938398358</v>
+      </c>
+      <c r="EZ4" t="n">
+        <v>0.1238262674119135</v>
+      </c>
+      <c r="FA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="FB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="FC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="FD4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="FE4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="FF4" t="n">
+        <v>4870</v>
+      </c>
+      <c r="FG4" t="n">
+        <v>23.26139630390144</v>
+      </c>
+      <c r="FH4" t="n">
+        <v>9.434887197387431</v>
+      </c>
+      <c r="FI4" t="n">
+        <v>1</v>
+      </c>
+      <c r="FJ4" t="n">
+        <v>17</v>
+      </c>
+      <c r="FK4" t="n">
+        <v>23</v>
+      </c>
+      <c r="FL4" t="n">
+        <v>29</v>
+      </c>
+      <c r="FM4" t="n">
+        <v>66</v>
+      </c>
+      <c r="FN4" t="n">
+        <v>4870</v>
+      </c>
+      <c r="FO4" t="n">
+        <v>68.50480492813142</v>
+      </c>
+      <c r="FP4" t="n">
+        <v>39.31157691569259</v>
+      </c>
+      <c r="FQ4" t="n">
+        <v>7</v>
+      </c>
+      <c r="FR4" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="FS4" t="n">
+        <v>58</v>
+      </c>
+      <c r="FT4" t="n">
+        <v>85.40000000000001</v>
+      </c>
+      <c r="FU4" t="n">
+        <v>319.4</v>
+      </c>
+      <c r="FV4" t="n">
+        <v>4870</v>
+      </c>
+      <c r="FW4" t="n">
         <v>0.5</v>
       </c>
-      <c r="ER4" t="n">
+      <c r="FX4" t="n">
         <v>0.5000513426093667</v>
       </c>
-      <c r="ES4" t="n">
-        <v>0</v>
-      </c>
-      <c r="ET4" t="n">
-        <v>0</v>
-      </c>
-      <c r="EU4" t="n">
+      <c r="FY4" t="n">
+        <v>0</v>
+      </c>
+      <c r="FZ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="GA4" t="n">
         <v>0.5</v>
       </c>
-      <c r="EV4" t="n">
-        <v>1</v>
-      </c>
-      <c r="EW4" t="n">
+      <c r="GB4" t="n">
+        <v>1</v>
+      </c>
+      <c r="GC4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2189,24 +2465,120 @@
         <v>4854</v>
       </c>
       <c r="EQ5" t="n">
+        <v>274.3298311444237</v>
+      </c>
+      <c r="ER5" t="n">
+        <v>25.47399486095894</v>
+      </c>
+      <c r="ES5" t="n">
+        <v>170.4000000059605</v>
+      </c>
+      <c r="ET5" t="n">
+        <v>257.000000089407</v>
+      </c>
+      <c r="EU5" t="n">
+        <v>274.1000000983477</v>
+      </c>
+      <c r="EV5" t="n">
+        <v>291.7500000819564</v>
+      </c>
+      <c r="EW5" t="n">
+        <v>367.000000089407</v>
+      </c>
+      <c r="EX5" t="n">
+        <v>4854</v>
+      </c>
+      <c r="EY5" t="n">
+        <v>0.08129377832715287</v>
+      </c>
+      <c r="EZ5" t="n">
+        <v>0.125438834126302</v>
+      </c>
+      <c r="FA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="FB5" t="n">
+        <v>0</v>
+      </c>
+      <c r="FC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="FD5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="FE5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="FF5" t="n">
+        <v>4854</v>
+      </c>
+      <c r="FG5" t="n">
+        <v>24.73856613102596</v>
+      </c>
+      <c r="FH5" t="n">
+        <v>9.930888735958241</v>
+      </c>
+      <c r="FI5" t="n">
+        <v>1</v>
+      </c>
+      <c r="FJ5" t="n">
+        <v>17</v>
+      </c>
+      <c r="FK5" t="n">
+        <v>24</v>
+      </c>
+      <c r="FL5" t="n">
+        <v>31</v>
+      </c>
+      <c r="FM5" t="n">
+        <v>72</v>
+      </c>
+      <c r="FN5" t="n">
+        <v>4854</v>
+      </c>
+      <c r="FO5" t="n">
+        <v>66.13081994231561</v>
+      </c>
+      <c r="FP5" t="n">
+        <v>39.0528751483616</v>
+      </c>
+      <c r="FQ5" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="FR5" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="FS5" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="FT5" t="n">
+        <v>82</v>
+      </c>
+      <c r="FU5" t="n">
+        <v>322</v>
+      </c>
+      <c r="FV5" t="n">
+        <v>4854</v>
+      </c>
+      <c r="FW5" t="n">
         <v>0.5</v>
       </c>
-      <c r="ER5" t="n">
+      <c r="FX5" t="n">
         <v>0.5000515118736235</v>
       </c>
-      <c r="ES5" t="n">
-        <v>0</v>
-      </c>
-      <c r="ET5" t="n">
-        <v>0</v>
-      </c>
-      <c r="EU5" t="n">
+      <c r="FY5" t="n">
+        <v>0</v>
+      </c>
+      <c r="FZ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="GA5" t="n">
         <v>0.5</v>
       </c>
-      <c r="EV5" t="n">
-        <v>1</v>
-      </c>
-      <c r="EW5" t="n">
+      <c r="GB5" t="n">
+        <v>1</v>
+      </c>
+      <c r="GC5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2652,24 +3024,120 @@
         <v>4938</v>
       </c>
       <c r="EQ6" t="n">
+        <v>269.2283718868541</v>
+      </c>
+      <c r="ER6" t="n">
+        <v>25.51109635866201</v>
+      </c>
+      <c r="ES6" t="n">
+        <v>184.200000077486</v>
+      </c>
+      <c r="ET6" t="n">
+        <v>252.0000000596046</v>
+      </c>
+      <c r="EU6" t="n">
+        <v>269.7500000596046</v>
+      </c>
+      <c r="EV6" t="n">
+        <v>287.0000000596046</v>
+      </c>
+      <c r="EW6" t="n">
+        <v>345.2000001072884</v>
+      </c>
+      <c r="EX6" t="n">
+        <v>4938</v>
+      </c>
+      <c r="EY6" t="n">
+        <v>0.07614418793033617</v>
+      </c>
+      <c r="EZ6" t="n">
+        <v>0.1220394060837249</v>
+      </c>
+      <c r="FA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="FB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="FC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="FD6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="FE6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="FF6" t="n">
+        <v>4938</v>
+      </c>
+      <c r="FG6" t="n">
+        <v>23.15350344268935</v>
+      </c>
+      <c r="FH6" t="n">
+        <v>9.733262947954556</v>
+      </c>
+      <c r="FI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="FJ6" t="n">
+        <v>16</v>
+      </c>
+      <c r="FK6" t="n">
+        <v>22</v>
+      </c>
+      <c r="FL6" t="n">
+        <v>29</v>
+      </c>
+      <c r="FM6" t="n">
+        <v>60</v>
+      </c>
+      <c r="FN6" t="n">
+        <v>4938</v>
+      </c>
+      <c r="FO6" t="n">
+        <v>66.14937221547184</v>
+      </c>
+      <c r="FP6" t="n">
+        <v>38.70591609383673</v>
+      </c>
+      <c r="FQ6" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="FR6" t="n">
+        <v>39.65</v>
+      </c>
+      <c r="FS6" t="n">
+        <v>57</v>
+      </c>
+      <c r="FT6" t="n">
+        <v>82.8</v>
+      </c>
+      <c r="FU6" t="n">
+        <v>370.2</v>
+      </c>
+      <c r="FV6" t="n">
+        <v>4938</v>
+      </c>
+      <c r="FW6" t="n">
         <v>0.5</v>
       </c>
-      <c r="ER6" t="n">
+      <c r="FX6" t="n">
         <v>0.5000506354753438</v>
       </c>
-      <c r="ES6" t="n">
-        <v>0</v>
-      </c>
-      <c r="ET6" t="n">
-        <v>0</v>
-      </c>
-      <c r="EU6" t="n">
+      <c r="FY6" t="n">
+        <v>0</v>
+      </c>
+      <c r="FZ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="GA6" t="n">
         <v>0.5</v>
       </c>
-      <c r="EV6" t="n">
-        <v>1</v>
-      </c>
-      <c r="EW6" t="n">
+      <c r="GB6" t="n">
+        <v>1</v>
+      </c>
+      <c r="GC6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3115,29 +3583,125 @@
         <v>4858</v>
       </c>
       <c r="EQ7" t="n">
+        <v>265.2878963279903</v>
+      </c>
+      <c r="ER7" t="n">
+        <v>25.25153517705949</v>
+      </c>
+      <c r="ES7" t="n">
+        <v>157.0000000596046</v>
+      </c>
+      <c r="ET7" t="n">
+        <v>249.0000000298023</v>
+      </c>
+      <c r="EU7" t="n">
+        <v>265.5250000804663</v>
+      </c>
+      <c r="EV7" t="n">
+        <v>282.000000089407</v>
+      </c>
+      <c r="EW7" t="n">
+        <v>345.000000089407</v>
+      </c>
+      <c r="EX7" t="n">
+        <v>4858</v>
+      </c>
+      <c r="EY7" t="n">
+        <v>0.09798270893371758</v>
+      </c>
+      <c r="EZ7" t="n">
+        <v>0.13810702237358</v>
+      </c>
+      <c r="FA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="FB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="FC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="FD7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="FE7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="FF7" t="n">
+        <v>4858</v>
+      </c>
+      <c r="FG7" t="n">
+        <v>27.49135446685879</v>
+      </c>
+      <c r="FH7" t="n">
+        <v>10.0539018459554</v>
+      </c>
+      <c r="FI7" t="n">
+        <v>2</v>
+      </c>
+      <c r="FJ7" t="n">
+        <v>20</v>
+      </c>
+      <c r="FK7" t="n">
+        <v>27</v>
+      </c>
+      <c r="FL7" t="n">
+        <v>34</v>
+      </c>
+      <c r="FM7" t="n">
+        <v>75</v>
+      </c>
+      <c r="FN7" t="n">
+        <v>4858</v>
+      </c>
+      <c r="FO7" t="n">
+        <v>69.37933305887196</v>
+      </c>
+      <c r="FP7" t="n">
+        <v>40.51733035502247</v>
+      </c>
+      <c r="FQ7" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="FR7" t="n">
+        <v>42</v>
+      </c>
+      <c r="FS7" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="FT7" t="n">
+        <v>86.15000000000001</v>
+      </c>
+      <c r="FU7" t="n">
+        <v>369.4</v>
+      </c>
+      <c r="FV7" t="n">
+        <v>4858</v>
+      </c>
+      <c r="FW7" t="n">
         <v>0.5</v>
       </c>
-      <c r="ER7" t="n">
+      <c r="FX7" t="n">
         <v>0.500051469453016</v>
       </c>
-      <c r="ES7" t="n">
-        <v>0</v>
-      </c>
-      <c r="ET7" t="n">
-        <v>0</v>
-      </c>
-      <c r="EU7" t="n">
+      <c r="FY7" t="n">
+        <v>0</v>
+      </c>
+      <c r="FZ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="GA7" t="n">
         <v>0.5</v>
       </c>
-      <c r="EV7" t="n">
-        <v>1</v>
-      </c>
-      <c r="EW7" t="n">
+      <c r="GB7" t="n">
+        <v>1</v>
+      </c>
+      <c r="GC7" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="23">
     <mergeCell ref="EH1:EO1"/>
     <mergeCell ref="EP1:EW1"/>
     <mergeCell ref="R1:Y1"/>
@@ -3147,13 +3711,17 @@
     <mergeCell ref="CT1:DA1"/>
     <mergeCell ref="BV1:CC1"/>
     <mergeCell ref="CD1:CK1"/>
+    <mergeCell ref="FF1:FM1"/>
     <mergeCell ref="DZ1:EG1"/>
+    <mergeCell ref="FN1:FU1"/>
     <mergeCell ref="AH1:AO1"/>
     <mergeCell ref="AP1:AW1"/>
     <mergeCell ref="B1:I1"/>
+    <mergeCell ref="EX1:FE1"/>
     <mergeCell ref="BN1:BU1"/>
     <mergeCell ref="DR1:DY1"/>
     <mergeCell ref="DJ1:DQ1"/>
+    <mergeCell ref="FV1:GC1"/>
     <mergeCell ref="Z1:AG1"/>
     <mergeCell ref="CL1:CS1"/>
     <mergeCell ref="BF1:BM1"/>

</xml_diff>